<commit_message>
Republish Prague_2025_WC: Kayak Cross individual (Time Trials) RANK from official classification (105 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Prague_2025_WC/Prague_2025_WC_start.xlsx
+++ b/events/Prague_2025_WC/Prague_2025_WC_start.xlsx
@@ -33779,6 +33779,11 @@
       <c r="K540" t="n">
         <v>539</v>
       </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R540" t="inlineStr">
         <is>
           <t>MILLS Waris</t>
@@ -33842,6 +33847,11 @@
       <c r="K541" t="n">
         <v>540</v>
       </c>
+      <c r="M541" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R541" t="inlineStr">
         <is>
           <t>WOOD Emmi</t>
@@ -33905,6 +33915,11 @@
       <c r="K542" t="n">
         <v>541</v>
       </c>
+      <c r="M542" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R542" t="inlineStr">
         <is>
           <t>LUKNAROVA Emanuela</t>
@@ -33968,6 +33983,11 @@
       <c r="K543" t="n">
         <v>542</v>
       </c>
+      <c r="M543" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R543" t="inlineStr">
         <is>
           <t>CHEN Lin</t>
@@ -34031,6 +34051,11 @@
       <c r="K544" t="n">
         <v>543</v>
       </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R544" t="inlineStr">
         <is>
           <t>NESNIDALOVA Lucie</t>
@@ -34094,6 +34119,11 @@
       <c r="K545" t="n">
         <v>544</v>
       </c>
+      <c r="M545" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R545" t="inlineStr">
         <is>
           <t>BAYN Nele</t>
@@ -34157,6 +34187,11 @@
       <c r="K546" t="n">
         <v>545</v>
       </c>
+      <c r="M546" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R546" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -34220,6 +34255,11 @@
       <c r="K547" t="n">
         <v>546</v>
       </c>
+      <c r="M547" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R547" t="inlineStr">
         <is>
           <t>WAN Shunfang</t>
@@ -34283,6 +34323,11 @@
       <c r="K548" t="n">
         <v>547</v>
       </c>
+      <c r="M548" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R548" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -34346,6 +34391,11 @@
       <c r="K549" t="n">
         <v>548</v>
       </c>
+      <c r="M549" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R549" t="inlineStr">
         <is>
           <t>GORA Aleksandra</t>
@@ -34472,6 +34522,11 @@
       <c r="K551" t="n">
         <v>550</v>
       </c>
+      <c r="M551" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R551" t="inlineStr">
         <is>
           <t>SORRIBES Laia</t>
@@ -34535,6 +34590,11 @@
       <c r="K552" t="n">
         <v>551</v>
       </c>
+      <c r="M552" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R552" t="inlineStr">
         <is>
           <t>WILLIAMS Courtney</t>
@@ -34598,6 +34658,11 @@
       <c r="K553" t="n">
         <v>552</v>
       </c>
+      <c r="M553" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R553" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -34661,6 +34726,11 @@
       <c r="K554" t="n">
         <v>553</v>
       </c>
+      <c r="M554" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R554" t="inlineStr">
         <is>
           <t>BALDONI Lea</t>
@@ -34724,6 +34794,11 @@
       <c r="K555" t="n">
         <v>554</v>
       </c>
+      <c r="M555" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R555" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -34787,6 +34862,11 @@
       <c r="K556" t="n">
         <v>555</v>
       </c>
+      <c r="M556" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R556" t="inlineStr">
         <is>
           <t>PANKOVA Zuzana</t>
@@ -34850,6 +34930,11 @@
       <c r="K557" t="n">
         <v>556</v>
       </c>
+      <c r="M557" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R557" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -34913,6 +34998,11 @@
       <c r="K558" t="n">
         <v>557</v>
       </c>
+      <c r="M558" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R558" t="inlineStr">
         <is>
           <t>NOVAK Ajda</t>
@@ -34976,6 +35066,11 @@
       <c r="K559" t="n">
         <v>558</v>
       </c>
+      <c r="M559" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R559" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -35039,6 +35134,11 @@
       <c r="K560" t="n">
         <v>559</v>
       </c>
+      <c r="M560" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R560" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -35102,6 +35202,11 @@
       <c r="K561" t="n">
         <v>560</v>
       </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R561" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -35165,6 +35270,11 @@
       <c r="K562" t="n">
         <v>561</v>
       </c>
+      <c r="M562" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R562" t="inlineStr">
         <is>
           <t>PINTERIC Naja</t>
@@ -35228,6 +35338,11 @@
       <c r="K563" t="n">
         <v>562</v>
       </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R563" t="inlineStr">
         <is>
           <t>BOUZIDI Carole</t>
@@ -35291,6 +35406,11 @@
       <c r="K564" t="n">
         <v>563</v>
       </c>
+      <c r="M564" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R564" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -35354,6 +35474,11 @@
       <c r="K565" t="n">
         <v>564</v>
       </c>
+      <c r="M565" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R565" t="inlineStr">
         <is>
           <t>XIE Xueting</t>
@@ -35417,6 +35542,11 @@
       <c r="K566" t="n">
         <v>565</v>
       </c>
+      <c r="M566" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R566" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -35480,6 +35610,11 @@
       <c r="K567" t="n">
         <v>566</v>
       </c>
+      <c r="M567" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R567" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -35543,6 +35678,11 @@
       <c r="K568" t="n">
         <v>567</v>
       </c>
+      <c r="M568" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R568" t="inlineStr">
         <is>
           <t>ZWOLINSKA Klaudia</t>
@@ -35606,6 +35746,11 @@
       <c r="K569" t="n">
         <v>568</v>
       </c>
+      <c r="M569" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R569" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -35669,6 +35814,11 @@
       <c r="K570" t="n">
         <v>569</v>
       </c>
+      <c r="M570" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R570" t="inlineStr">
         <is>
           <t>FOX Jessica</t>
@@ -35732,6 +35882,11 @@
       <c r="K571" t="n">
         <v>570</v>
       </c>
+      <c r="M571" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R571" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -35795,6 +35950,11 @@
       <c r="K572" t="n">
         <v>571</v>
       </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R572" t="inlineStr">
         <is>
           <t>LILIK Elena</t>
@@ -35858,6 +36018,11 @@
       <c r="K573" t="n">
         <v>572</v>
       </c>
+      <c r="M573" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R573" t="inlineStr">
         <is>
           <t>VUITTON Emma</t>
@@ -35921,6 +36086,11 @@
       <c r="K574" t="n">
         <v>573</v>
       </c>
+      <c r="M574" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R574" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -35984,6 +36154,11 @@
       <c r="K575" t="n">
         <v>574</v>
       </c>
+      <c r="M575" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R575" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -36047,6 +36222,11 @@
       <c r="K576" t="n">
         <v>575</v>
       </c>
+      <c r="M576" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R576" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -36110,6 +36290,11 @@
       <c r="K577" t="n">
         <v>576</v>
       </c>
+      <c r="M577" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R577" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -36173,6 +36358,11 @@
       <c r="K578" t="n">
         <v>577</v>
       </c>
+      <c r="M578" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R578" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -36236,6 +36426,11 @@
       <c r="K579" t="n">
         <v>578</v>
       </c>
+      <c r="M579" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R579" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -36299,6 +36494,11 @@
       <c r="K580" t="n">
         <v>579</v>
       </c>
+      <c r="M580" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R580" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -36362,6 +36562,11 @@
       <c r="K581" t="n">
         <v>580</v>
       </c>
+      <c r="M581" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R581" t="inlineStr">
         <is>
           <t>WOODS Kimberley</t>
@@ -36425,6 +36630,11 @@
       <c r="K582" t="n">
         <v>581</v>
       </c>
+      <c r="M582" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R582" t="inlineStr">
         <is>
           <t>EIGEL Pavel</t>
@@ -36488,6 +36698,11 @@
       <c r="K583" t="n">
         <v>582</v>
       </c>
+      <c r="M583" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="R583" t="inlineStr">
         <is>
           <t>RAW Brayden</t>
@@ -36551,6 +36766,11 @@
       <c r="K584" t="n">
         <v>583</v>
       </c>
+      <c r="M584" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="R584" t="inlineStr">
         <is>
           <t>VAN HEERDEN Matthew</t>
@@ -36614,6 +36834,11 @@
       <c r="K585" t="n">
         <v>584</v>
       </c>
+      <c r="M585" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R585" t="inlineStr">
         <is>
           <t>MUTO Yusuke</t>
@@ -36677,6 +36902,11 @@
       <c r="K586" t="n">
         <v>585</v>
       </c>
+      <c r="M586" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R586" t="inlineStr">
         <is>
           <t>TEMIRGALIEV Djanibek</t>
@@ -36740,6 +36970,11 @@
       <c r="K587" t="n">
         <v>586</v>
       </c>
+      <c r="M587" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R587" t="inlineStr">
         <is>
           <t>MING Xingzhou</t>
@@ -36803,6 +37038,11 @@
       <c r="K588" t="n">
         <v>587</v>
       </c>
+      <c r="M588" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R588" t="inlineStr">
         <is>
           <t>MAPELLI Guilherme</t>
@@ -36866,6 +37106,11 @@
       <c r="K589" t="n">
         <v>588</v>
       </c>
+      <c r="M589" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R589" t="inlineStr">
         <is>
           <t>ZHANG Hejie</t>
@@ -36929,6 +37174,11 @@
       <c r="K590" t="n">
         <v>589</v>
       </c>
+      <c r="M590" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R590" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -36992,6 +37242,11 @@
       <c r="K591" t="n">
         <v>590</v>
       </c>
+      <c r="M591" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R591" t="inlineStr">
         <is>
           <t>GONSENICA Adam</t>
@@ -37055,6 +37310,11 @@
       <c r="K592" t="n">
         <v>591</v>
       </c>
+      <c r="M592" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="R592" t="inlineStr">
         <is>
           <t>MAGAN Raage</t>
@@ -37118,6 +37378,11 @@
       <c r="K593" t="n">
         <v>592</v>
       </c>
+      <c r="M593" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R593" t="inlineStr">
         <is>
           <t>MAGAN Aar</t>
@@ -37181,6 +37446,11 @@
       <c r="K594" t="n">
         <v>593</v>
       </c>
+      <c r="M594" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="R594" t="inlineStr">
         <is>
           <t>TANAKA Yuuki</t>
@@ -37244,6 +37514,11 @@
       <c r="K595" t="n">
         <v>594</v>
       </c>
+      <c r="M595" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R595" t="inlineStr">
         <is>
           <t>ZEITLHOFER Simon</t>
@@ -37370,6 +37645,11 @@
       <c r="K597" t="n">
         <v>596</v>
       </c>
+      <c r="M597" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R597" t="inlineStr">
         <is>
           <t>GRIGAR Jakub</t>
@@ -37433,6 +37713,11 @@
       <c r="K598" t="n">
         <v>597</v>
       </c>
+      <c r="M598" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R598" t="inlineStr">
         <is>
           <t>ROZENTALS Klass Francisks</t>
@@ -37496,6 +37781,11 @@
       <c r="K599" t="n">
         <v>598</v>
       </c>
+      <c r="M599" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="R599" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -37622,6 +37912,11 @@
       <c r="K601" t="n">
         <v>600</v>
       </c>
+      <c r="M601" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R601" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -37685,6 +37980,11 @@
       <c r="K602" t="n">
         <v>601</v>
       </c>
+      <c r="M602" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R602" t="inlineStr">
         <is>
           <t>HUANG Liman</t>
@@ -37748,6 +38048,11 @@
       <c r="K603" t="n">
         <v>602</v>
       </c>
+      <c r="M603" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R603" t="inlineStr">
         <is>
           <t>ZIELONKA Mark</t>
@@ -37811,6 +38116,11 @@
       <c r="K604" t="n">
         <v>603</v>
       </c>
+      <c r="M604" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R604" t="inlineStr">
         <is>
           <t>BOYD Trevor</t>
@@ -37874,6 +38184,11 @@
       <c r="K605" t="n">
         <v>604</v>
       </c>
+      <c r="M605" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R605" t="inlineStr">
         <is>
           <t>PUCHNER Oliver</t>
@@ -37937,6 +38252,11 @@
       <c r="K606" t="n">
         <v>605</v>
       </c>
+      <c r="M606" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="R606" t="inlineStr">
         <is>
           <t>TRIPANO Manuel</t>
@@ -38000,6 +38320,11 @@
       <c r="K607" t="n">
         <v>606</v>
       </c>
+      <c r="M607" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R607" t="inlineStr">
         <is>
           <t>BRZEZINSKI Jakub</t>
@@ -38063,6 +38388,11 @@
       <c r="K608" t="n">
         <v>607</v>
       </c>
+      <c r="M608" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="R608" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -38126,6 +38456,11 @@
       <c r="K609" t="n">
         <v>608</v>
       </c>
+      <c r="M609" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R609" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -38189,6 +38524,11 @@
       <c r="K610" t="n">
         <v>609</v>
       </c>
+      <c r="M610" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R610" t="inlineStr">
         <is>
           <t>AUBERTIN Maxime</t>
@@ -38252,6 +38592,11 @@
       <c r="K611" t="n">
         <v>610</v>
       </c>
+      <c r="M611" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R611" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -38315,6 +38660,11 @@
       <c r="K612" t="n">
         <v>611</v>
       </c>
+      <c r="M612" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R612" t="inlineStr">
         <is>
           <t>PASIUT Michal</t>
@@ -38378,6 +38728,11 @@
       <c r="K613" t="n">
         <v>612</v>
       </c>
+      <c r="M613" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R613" t="inlineStr">
         <is>
           <t>MARTINEZ Jesus</t>
@@ -38441,6 +38796,11 @@
       <c r="K614" t="n">
         <v>613</v>
       </c>
+      <c r="M614" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R614" t="inlineStr">
         <is>
           <t>KUDER MARUSIC Vid</t>
@@ -38504,6 +38864,11 @@
       <c r="K615" t="n">
         <v>614</v>
       </c>
+      <c r="M615" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="R615" t="inlineStr">
         <is>
           <t>MCCREERY Alistair</t>
@@ -38630,6 +38995,11 @@
       <c r="K617" t="n">
         <v>616</v>
       </c>
+      <c r="M617" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R617" t="inlineStr">
         <is>
           <t>COLLIER Nicholas</t>
@@ -38693,6 +39063,11 @@
       <c r="K618" t="n">
         <v>617</v>
       </c>
+      <c r="M618" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R618" t="inlineStr">
         <is>
           <t>POPE Benjamin</t>
@@ -38756,6 +39131,11 @@
       <c r="K619" t="n">
         <v>618</v>
       </c>
+      <c r="M619" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R619" t="inlineStr">
         <is>
           <t>ROELLER Tillmann</t>
@@ -38819,6 +39199,11 @@
       <c r="K620" t="n">
         <v>619</v>
       </c>
+      <c r="M620" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R620" t="inlineStr">
         <is>
           <t>KANCLER Tine</t>
@@ -38882,6 +39267,11 @@
       <c r="K621" t="n">
         <v>620</v>
       </c>
+      <c r="M621" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R621" t="inlineStr">
         <is>
           <t>OHRSTROM Isak</t>
@@ -38945,6 +39335,11 @@
       <c r="K622" t="n">
         <v>621</v>
       </c>
+      <c r="M622" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R622" t="inlineStr">
         <is>
           <t>LONG Kyler James</t>
@@ -39071,6 +39466,11 @@
       <c r="K624" t="n">
         <v>623</v>
       </c>
+      <c r="M624" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R624" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -39134,6 +39534,11 @@
       <c r="K625" t="n">
         <v>624</v>
       </c>
+      <c r="M625" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R625" t="inlineStr">
         <is>
           <t>DE COSTER Gabriel</t>
@@ -39197,6 +39602,11 @@
       <c r="K626" t="n">
         <v>625</v>
       </c>
+      <c r="M626" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R626" t="inlineStr">
         <is>
           <t>CHIARELLO Gelindo</t>
@@ -39260,6 +39670,11 @@
       <c r="K627" t="n">
         <v>626</v>
       </c>
+      <c r="M627" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R627" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -39323,6 +39738,11 @@
       <c r="K628" t="n">
         <v>627</v>
       </c>
+      <c r="M628" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R628" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -39386,6 +39806,11 @@
       <c r="K629" t="n">
         <v>628</v>
       </c>
+      <c r="M629" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R629" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -39449,6 +39874,11 @@
       <c r="K630" t="n">
         <v>629</v>
       </c>
+      <c r="M630" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R630" t="inlineStr">
         <is>
           <t>HOLMER Erik</t>
@@ -39512,6 +39942,11 @@
       <c r="K631" t="n">
         <v>630</v>
       </c>
+      <c r="M631" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
       <c r="R631" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -39575,6 +40010,11 @@
       <c r="K632" t="n">
         <v>631</v>
       </c>
+      <c r="M632" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R632" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -39638,6 +40078,11 @@
       <c r="K633" t="n">
         <v>632</v>
       </c>
+      <c r="M633" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R633" t="inlineStr">
         <is>
           <t>CASTRYCK Titouan</t>
@@ -39701,6 +40146,11 @@
       <c r="K634" t="n">
         <v>633</v>
       </c>
+      <c r="M634" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R634" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -39764,6 +40214,11 @@
       <c r="K635" t="n">
         <v>634</v>
       </c>
+      <c r="M635" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R635" t="inlineStr">
         <is>
           <t>ANDERSON Timothy</t>
@@ -39827,6 +40282,11 @@
       <c r="K636" t="n">
         <v>635</v>
       </c>
+      <c r="M636" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R636" t="inlineStr">
         <is>
           <t>DICKSON Jonny</t>
@@ -39890,6 +40350,11 @@
       <c r="K637" t="n">
         <v>636</v>
       </c>
+      <c r="M637" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R637" t="inlineStr">
         <is>
           <t>ECHEVERRIA OLGUIN Andraz</t>
@@ -39953,6 +40418,11 @@
       <c r="K638" t="n">
         <v>637</v>
       </c>
+      <c r="M638" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R638" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -40016,6 +40486,11 @@
       <c r="K639" t="n">
         <v>638</v>
       </c>
+      <c r="M639" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R639" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -40079,6 +40554,11 @@
       <c r="K640" t="n">
         <v>639</v>
       </c>
+      <c r="M640" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R640" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -40142,6 +40622,11 @@
       <c r="K641" t="n">
         <v>640</v>
       </c>
+      <c r="M641" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R641" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -40205,6 +40690,11 @@
       <c r="K642" t="n">
         <v>641</v>
       </c>
+      <c r="M642" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R642" t="inlineStr">
         <is>
           <t>HEGGE Noah</t>
@@ -40268,6 +40758,11 @@
       <c r="K643" t="n">
         <v>642</v>
       </c>
+      <c r="M643" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R643" t="inlineStr">
         <is>
           <t>DE GENNARO Giovanni</t>
@@ -40331,6 +40826,11 @@
       <c r="K644" t="n">
         <v>643</v>
       </c>
+      <c r="M644" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R644" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -40394,6 +40894,11 @@
       <c r="K645" t="n">
         <v>644</v>
       </c>
+      <c r="M645" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R645" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -40457,6 +40962,11 @@
       <c r="K646" t="n">
         <v>645</v>
       </c>
+      <c r="M646" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R646" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -40520,6 +41030,11 @@
       <c r="K647" t="n">
         <v>646</v>
       </c>
+      <c r="M647" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R647" t="inlineStr">
         <is>
           <t>DOUGOUD Martin</t>
@@ -40583,6 +41098,11 @@
       <c r="K648" t="n">
         <v>647</v>
       </c>
+      <c r="M648" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R648" t="inlineStr">
         <is>
           <t>BUTCHER Finn</t>
@@ -40645,6 +41165,11 @@
       </c>
       <c r="K649" t="n">
         <v>648</v>
+      </c>
+      <c r="M649" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="R649" t="inlineStr">
         <is>

</xml_diff>